<commit_message>
Show the NSE index itself in the survivorship sheet
Rows 5 and 6 are now the CAGR and MaxDD of each universe's own NSE index
file (close column, 2019-01-01 to 2026-05-29). These files are price indices,
not total-return indices, which the docstring states. The equal-weight
basket moves to two rows at the end, still checked against the published buy
& hold figures.

The CSV is now written with the csv module: two labels contain commas, and
the joined lines split each into an extra column.
</commit_message>
<xml_diff>
--- a/diagnostics/survivorship_sheet_research.xlsx
+++ b/diagnostics/survivorship_sheet_research.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -694,104 +694,104 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>reference index: CAGR</t>
+          <t>NSE index: CAGR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>26.56</t>
+          <t>16.99</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>24.94</t>
+          <t>18.70</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>26.25</t>
+          <t>18.20</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>23.72</t>
+          <t>18.66</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>25.60</t>
+          <t>12.94</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>25.12</t>
+          <t>12.34</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>23.91</t>
+          <t>11.28</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>20.45</t>
+          <t>10.95</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>27.89</t>
+          <t>21.27</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>reference index: MaxDD</t>
+          <t>NSE index: MaxDD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-48.95</t>
+          <t>-46.31</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>-37.67</t>
+          <t>-38.67</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-38.89</t>
+          <t>-40.16</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-37.92</t>
+          <t>-43.07</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>-41.56</t>
+          <t>-38.30</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-38.03</t>
+          <t>-38.22</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>-37.40</t>
+          <t>-38.10</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>-37.31</t>
+          <t>-38.44</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>-48.60</t>
+          <t>-57.47</t>
         </is>
       </c>
     </row>
@@ -1000,6 +1000,110 @@
       <c r="J11" t="inlineStr">
         <is>
           <t>-7.86 (from 2021-10-29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>equal-weight basket (untaxed, daily rebalanced): CAGR</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>26.56</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>24.94</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>26.25</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>23.72</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>25.60</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>25.12</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>23.91</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>20.45</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>27.89</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>equal-weight basket (untaxed, daily rebalanced): MaxDD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>-48.95</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>-37.67</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>-38.89</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>-37.92</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>-41.56</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-38.03</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>-37.40</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>-37.31</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>-48.60</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1280,104 +1384,104 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>reference index: CAGR</t>
+          <t>NSE index: CAGR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>26.56</t>
+          <t>16.99</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>24.94</t>
+          <t>18.70</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>26.25</t>
+          <t>18.20</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>23.72</t>
+          <t>18.66</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>25.60</t>
+          <t>12.94</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>25.12</t>
+          <t>12.34</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>23.91</t>
+          <t>11.28</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>20.45</t>
+          <t>10.95</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>27.89</t>
+          <t>21.27</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>reference index: MaxDD</t>
+          <t>NSE index: MaxDD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-48.95</t>
+          <t>-46.31</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>-37.67</t>
+          <t>-38.67</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-38.89</t>
+          <t>-40.16</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-37.92</t>
+          <t>-43.07</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>-41.56</t>
+          <t>-38.30</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-38.03</t>
+          <t>-38.22</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>-37.40</t>
+          <t>-38.10</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>-37.31</t>
+          <t>-38.44</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>-48.60</t>
+          <t>-57.47</t>
         </is>
       </c>
     </row>
@@ -1586,6 +1690,110 @@
       <c r="J11" t="inlineStr">
         <is>
           <t>-4.09 (from 2021-10-29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>equal-weight basket (untaxed, daily rebalanced): CAGR</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>26.56</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>24.94</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>26.25</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>23.72</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>25.60</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>25.12</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>23.91</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>20.45</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>27.89</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>equal-weight basket (untaxed, daily rebalanced): MaxDD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>-48.95</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>-37.67</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>-38.89</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>-37.92</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>-41.56</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-38.03</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>-37.40</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>-37.31</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>-48.60</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1866,104 +2074,104 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>reference index: CAGR</t>
+          <t>NSE index: CAGR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>26.56</t>
+          <t>16.99</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>24.94</t>
+          <t>18.70</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>26.25</t>
+          <t>18.20</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>23.72</t>
+          <t>18.66</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>25.60</t>
+          <t>12.94</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>25.12</t>
+          <t>12.34</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>23.91</t>
+          <t>11.28</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>20.45</t>
+          <t>10.95</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>27.89</t>
+          <t>21.27</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>reference index: MaxDD</t>
+          <t>NSE index: MaxDD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-48.95</t>
+          <t>-46.31</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>-37.67</t>
+          <t>-38.67</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-38.89</t>
+          <t>-40.16</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-37.92</t>
+          <t>-43.07</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>-41.56</t>
+          <t>-38.30</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-38.03</t>
+          <t>-38.22</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>-37.40</t>
+          <t>-38.10</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>-37.31</t>
+          <t>-38.44</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>-48.60</t>
+          <t>-57.47</t>
         </is>
       </c>
     </row>
@@ -2172,6 +2380,110 @@
       <c r="J11" t="inlineStr">
         <is>
           <t>-8.43 (from 2021-10-29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>equal-weight basket (untaxed, daily rebalanced): CAGR</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>26.56</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>24.94</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>26.25</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>23.72</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>25.60</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>25.12</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>23.91</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>20.45</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>27.89</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>equal-weight basket (untaxed, daily rebalanced): MaxDD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>-48.95</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>-37.67</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>-38.89</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>-37.92</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>-41.56</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-38.03</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>-37.40</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>-37.31</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>-48.60</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2452,104 +2764,104 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>reference index: CAGR</t>
+          <t>NSE index: CAGR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>26.56</t>
+          <t>16.99</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>24.94</t>
+          <t>18.70</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>26.25</t>
+          <t>18.20</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>23.72</t>
+          <t>18.66</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>25.60</t>
+          <t>12.94</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>25.12</t>
+          <t>12.34</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>23.91</t>
+          <t>11.28</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>20.45</t>
+          <t>10.95</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>27.89</t>
+          <t>21.27</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>reference index: MaxDD</t>
+          <t>NSE index: MaxDD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-48.95</t>
+          <t>-46.31</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>-37.67</t>
+          <t>-38.67</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-38.89</t>
+          <t>-40.16</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-37.92</t>
+          <t>-43.07</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>-41.56</t>
+          <t>-38.30</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>-38.03</t>
+          <t>-38.22</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>-37.40</t>
+          <t>-38.10</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>-37.31</t>
+          <t>-38.44</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>-48.60</t>
+          <t>-57.47</t>
         </is>
       </c>
     </row>
@@ -2758,6 +3070,110 @@
       <c r="J11" t="inlineStr">
         <is>
           <t>-5.04 (from 2021-10-29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>equal-weight basket (untaxed, daily rebalanced): CAGR</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>26.56</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>24.94</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>26.25</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>23.72</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>25.60</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>25.12</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>23.91</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>20.45</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>27.89</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>equal-weight basket (untaxed, daily rebalanced): MaxDD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>-48.95</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>-37.67</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>-38.89</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>-37.92</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>-41.56</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-38.03</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>-37.40</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>-37.31</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>-48.60</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild the survivorship sheet and the GATE 9 diagnostics for twelve universes
survivorship_sheet_research.csv and .xlsx are rebuilt from d961127 with the three
market-cap columns after microcap250. Every static CAGR and MaxDD was checked
against v34_comparison by the script. The pit rows read "not available: no
membership file for this supplier bucket", and a NOTES block carries the bias
label. The nine existing columns are identical to the previous file in the CSV and
on every sheet of the xlsx.

checkB_execution_timing.txt, leakage_check1_causality.txt and
leakage_check2_trading_purge.txt are the GATE 9 delegates' outputs from the
check_all run on d961127. Each gains the three universes' blocks, and its summary
line now counts 12 universes.
</commit_message>
<xml_diff>
--- a/diagnostics/survivorship_sheet_research.xlsx
+++ b/diagnostics/survivorship_sheet_research.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,6 +482,21 @@
           <t>microcap250</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>mcap1500to5000</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>mcap5001to10000</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>mcapover10000</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -534,6 +549,21 @@
           <t>30.00 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -586,6 +616,21 @@
           <t>25.15 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -638,6 +683,21 @@
           <t>53.07</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>54.03</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>62.82</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>48.71</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -690,6 +750,21 @@
           <t>43.30</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>44.31</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>53.28</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>41.05</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -742,6 +817,21 @@
           <t>21.27</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>12.94</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>12.94</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>12.94</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -794,6 +884,21 @@
           <t>-57.47</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>-38.30</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>-38.30</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>-38.30</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -846,6 +951,21 @@
           <t>-42.45</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>-41.52</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>-34.26</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>-32.59</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -898,6 +1018,21 @@
           <t>-6.51</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>-6.33</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>-4.39</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>-4.61</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -950,6 +1085,21 @@
           <t>-31.54 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1002,6 +1152,21 @@
           <t>-7.86 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -1054,6 +1219,21 @@
           <t>27.89</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>146.88</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>28.67</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>25.29</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1104,6 +1284,69 @@
       <c r="J13" t="inlineStr">
         <is>
           <t>-48.60</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>-49.75</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>-48.69</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>-40.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>row</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>NOTE mcap1500to5000</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>STATIC AND NOT AN INDEX. The supplier delivered these 478 names as a market-cap bucket, with no membership history. Only 2 of the 478 stop trading before the window ends, so the list appears to hold the bucket's members near the time of delivery, not the members at each date. A stock that left the bucket or was delisted is likely missing; a stock that grew into it is present for the whole window. Both the strategy and its buy &amp; hold therefore likely carry survivorship and look-ahead bias, which cannot be measured without membership files. The benchmark index is the broad NIFTY 500, not a bucket index.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NOTE mcap5001to10000</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>STATIC AND NOT AN INDEX. The supplier delivered these 216 names as a market-cap bucket, with no membership history. Only 0 of the 216 stop trading before the window ends, so the list appears to hold the bucket's members near the time of delivery, not the members at each date. A stock that left the bucket or was delisted is likely missing; a stock that grew into it is present for the whole window. Both the strategy and its buy &amp; hold therefore likely carry survivorship and look-ahead bias, which cannot be measured without membership files. The benchmark index is the broad NIFTY 500, not a bucket index.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>NOTE mcapover10000</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>STATIC AND NOT AN INDEX. The supplier delivered these 538 names as a market-cap bucket, with no membership history. Only 2 of the 538 stop trading before the window ends, so the list appears to hold the bucket's members near the time of delivery, not the members at each date. A stock that left the bucket or was delisted is likely missing; a stock that grew into it is present for the whole window. Both the strategy and its buy &amp; hold therefore likely carry survivorship and look-ahead bias, which cannot be measured without membership files. The benchmark index is the broad NIFTY 500, not a bucket index.</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1172,6 +1415,21 @@
           <t>microcap250</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>mcap1500to5000</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>mcap5001to10000</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>mcapover10000</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -1224,6 +1482,21 @@
           <t>21.46 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -1276,6 +1549,21 @@
           <t>18.04 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -1328,6 +1616,21 @@
           <t>32.11</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>27.82</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>39.04</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>32.77</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -1380,6 +1683,21 @@
           <t>26.90</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>23.46</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>32.70</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>27.66</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -1432,6 +1750,21 @@
           <t>21.27</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>12.94</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>12.94</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>12.94</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -1484,6 +1817,21 @@
           <t>-57.47</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>-38.30</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>-38.30</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>-38.30</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -1536,6 +1884,21 @@
           <t>-22.63</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>-21.92</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>-20.88</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>-18.59</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -1588,6 +1951,21 @@
           <t>-3.71</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>-4.67</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>-3.22</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>-3.01</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -1640,6 +2018,21 @@
           <t>-13.56 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1692,6 +2085,21 @@
           <t>-4.09 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -1744,6 +2152,21 @@
           <t>27.89</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>146.88</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>28.67</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>25.29</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1794,6 +2217,69 @@
       <c r="J13" t="inlineStr">
         <is>
           <t>-48.60</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>-49.75</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>-48.69</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>-40.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>row</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>NOTE mcap1500to5000</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>STATIC AND NOT AN INDEX. The supplier delivered these 478 names as a market-cap bucket, with no membership history. Only 2 of the 478 stop trading before the window ends, so the list appears to hold the bucket's members near the time of delivery, not the members at each date. A stock that left the bucket or was delisted is likely missing; a stock that grew into it is present for the whole window. Both the strategy and its buy &amp; hold therefore likely carry survivorship and look-ahead bias, which cannot be measured without membership files. The benchmark index is the broad NIFTY 500, not a bucket index.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NOTE mcap5001to10000</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>STATIC AND NOT AN INDEX. The supplier delivered these 216 names as a market-cap bucket, with no membership history. Only 0 of the 216 stop trading before the window ends, so the list appears to hold the bucket's members near the time of delivery, not the members at each date. A stock that left the bucket or was delisted is likely missing; a stock that grew into it is present for the whole window. Both the strategy and its buy &amp; hold therefore likely carry survivorship and look-ahead bias, which cannot be measured without membership files. The benchmark index is the broad NIFTY 500, not a bucket index.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>NOTE mcapover10000</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>STATIC AND NOT AN INDEX. The supplier delivered these 538 names as a market-cap bucket, with no membership history. Only 2 of the 538 stop trading before the window ends, so the list appears to hold the bucket's members near the time of delivery, not the members at each date. A stock that left the bucket or was delisted is likely missing; a stock that grew into it is present for the whole window. Both the strategy and its buy &amp; hold therefore likely carry survivorship and look-ahead bias, which cannot be measured without membership files. The benchmark index is the broad NIFTY 500, not a bucket index.</t>
         </is>
       </c>
     </row>
@@ -1808,7 +2294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1862,6 +2348,21 @@
           <t>microcap250</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>mcap1500to5000</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>mcap5001to10000</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>mcapover10000</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -1914,6 +2415,21 @@
           <t>37.07 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -1966,6 +2482,21 @@
           <t>30.54 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -2018,6 +2549,21 @@
           <t>67.11</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>58.54</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>53.65</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>53.22</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -2070,6 +2616,21 @@
           <t>55.53</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>49.82</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>46.45</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>44.94</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -2122,6 +2683,21 @@
           <t>21.27</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>12.94</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>12.94</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>12.94</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -2174,6 +2750,21 @@
           <t>-57.47</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>-38.30</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>-38.30</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>-38.30</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -2226,6 +2817,21 @@
           <t>-40.97</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>-50.93</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>-38.72</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>-35.21</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -2278,6 +2884,21 @@
           <t>-8.43</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>-7.90</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>-8.09</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>-6.65</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -2330,6 +2951,21 @@
           <t>-32.46 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -2382,6 +3018,21 @@
           <t>-8.43 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -2434,6 +3085,21 @@
           <t>27.89</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>146.88</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>28.67</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>25.29</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -2484,6 +3150,69 @@
       <c r="J13" t="inlineStr">
         <is>
           <t>-48.60</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>-49.75</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>-48.69</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>-40.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>row</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>NOTE mcap1500to5000</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>STATIC AND NOT AN INDEX. The supplier delivered these 478 names as a market-cap bucket, with no membership history. Only 2 of the 478 stop trading before the window ends, so the list appears to hold the bucket's members near the time of delivery, not the members at each date. A stock that left the bucket or was delisted is likely missing; a stock that grew into it is present for the whole window. Both the strategy and its buy &amp; hold therefore likely carry survivorship and look-ahead bias, which cannot be measured without membership files. The benchmark index is the broad NIFTY 500, not a bucket index.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NOTE mcap5001to10000</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>STATIC AND NOT AN INDEX. The supplier delivered these 216 names as a market-cap bucket, with no membership history. Only 0 of the 216 stop trading before the window ends, so the list appears to hold the bucket's members near the time of delivery, not the members at each date. A stock that left the bucket or was delisted is likely missing; a stock that grew into it is present for the whole window. Both the strategy and its buy &amp; hold therefore likely carry survivorship and look-ahead bias, which cannot be measured without membership files. The benchmark index is the broad NIFTY 500, not a bucket index.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>NOTE mcapover10000</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>STATIC AND NOT AN INDEX. The supplier delivered these 538 names as a market-cap bucket, with no membership history. Only 2 of the 538 stop trading before the window ends, so the list appears to hold the bucket's members near the time of delivery, not the members at each date. A stock that left the bucket or was delisted is likely missing; a stock that grew into it is present for the whole window. Both the strategy and its buy &amp; hold therefore likely carry survivorship and look-ahead bias, which cannot be measured without membership files. The benchmark index is the broad NIFTY 500, not a bucket index.</t>
         </is>
       </c>
     </row>
@@ -2498,7 +3227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2552,6 +3281,21 @@
           <t>microcap250</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>mcap1500to5000</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>mcap5001to10000</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>mcapover10000</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -2604,6 +3348,21 @@
           <t>30.07 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -2656,6 +3415,21 @@
           <t>25.17 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -2708,6 +3482,21 @@
           <t>39.41</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>30.59</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>37.83</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>34.87</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -2760,6 +3549,21 @@
           <t>33.08</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>25.78</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>31.88</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>29.62</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -2812,6 +3616,21 @@
           <t>21.27</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>12.94</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>12.94</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>12.94</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -2864,6 +3683,21 @@
           <t>-57.47</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>-38.30</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>-38.30</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>-38.30</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -2916,6 +3750,21 @@
           <t>-20.61</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>-31.29</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>-24.68</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>-22.05</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -2968,6 +3817,21 @@
           <t>-5.25</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>-5.44</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>-5.05</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>-4.72</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -3020,6 +3884,21 @@
           <t>-17.93 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -3072,6 +3951,21 @@
           <t>-5.04 (from 2021-10-29)</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>not available: no membership file for this supplier bucket</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -3124,6 +4018,21 @@
           <t>27.89</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>146.88</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>28.67</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>25.29</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -3174,6 +4083,69 @@
       <c r="J13" t="inlineStr">
         <is>
           <t>-48.60</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>-49.75</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>-48.69</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>-40.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>row</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>NOTE mcap1500to5000</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>STATIC AND NOT AN INDEX. The supplier delivered these 478 names as a market-cap bucket, with no membership history. Only 2 of the 478 stop trading before the window ends, so the list appears to hold the bucket's members near the time of delivery, not the members at each date. A stock that left the bucket or was delisted is likely missing; a stock that grew into it is present for the whole window. Both the strategy and its buy &amp; hold therefore likely carry survivorship and look-ahead bias, which cannot be measured without membership files. The benchmark index is the broad NIFTY 500, not a bucket index.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NOTE mcap5001to10000</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>STATIC AND NOT AN INDEX. The supplier delivered these 216 names as a market-cap bucket, with no membership history. Only 0 of the 216 stop trading before the window ends, so the list appears to hold the bucket's members near the time of delivery, not the members at each date. A stock that left the bucket or was delisted is likely missing; a stock that grew into it is present for the whole window. Both the strategy and its buy &amp; hold therefore likely carry survivorship and look-ahead bias, which cannot be measured without membership files. The benchmark index is the broad NIFTY 500, not a bucket index.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>NOTE mcapover10000</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>STATIC AND NOT AN INDEX. The supplier delivered these 538 names as a market-cap bucket, with no membership history. Only 2 of the 538 stop trading before the window ends, so the list appears to hold the bucket's members near the time of delivery, not the members at each date. A stock that left the bucket or was delisted is likely missing; a stock that grew into it is present for the whole window. Both the strategy and its buy &amp; hold therefore likely carry survivorship and look-ahead bias, which cannot be measured without membership files. The benchmark index is the broad NIFTY 500, not a bucket index.</t>
         </is>
       </c>
     </row>

</xml_diff>